<commit_message>
judge_cloud: an error is scored as an error, not invented (a not_on_site question with an error counted as invented in the 21/10 morning run); the summary lists invented separately
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/eval_answers_voyage.xlsx
+++ b/data/eval_answers_voyage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Phoenix\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8AA22F33-0AEA-48CC-A6A0-C1784C0432B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{1ED266BD-43D4-47CD-A9A7-36DAE479B0FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{23D1F696-CE00-4280-92FA-73F832BE444F}"/>
   </bookViews>
@@ -1361,6 +1361,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE116045-8EBF-452F-AC9A-A94C05B6A648}">
   <dimension ref="A1:L36"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="57.25" customWidth="1"/>
+    <col min="9" max="9" width="1.75" customWidth="1"/>
+    <col min="10" max="11" width="8.6640625" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="45.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>